<commit_message>
staff summary building files from template
</commit_message>
<xml_diff>
--- a/XcelUnify/Data/staff-summary.xlsx
+++ b/XcelUnify/Data/staff-summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_work\melb\2025\safe\Application\XcelUnify\XcelUnify\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69FE85BE-689E-4F5A-B985-E1DED515723C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1FE73A-E430-4252-800C-8C5883DA3CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{D83A47D0-BE84-4F4B-BC6D-31D7CF1B83A6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="31">
   <si>
     <t>Name</t>
   </si>
@@ -138,6 +138,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -253,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -270,6 +273,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -720,110 +724,113 @@
       <c r="B9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="12">
         <v>1</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="12">
         <v>6</v>
       </c>
-      <c r="E9" s="7">
-        <v>0</v>
-      </c>
-      <c r="F9" s="7">
+      <c r="E9" s="12">
+        <v>0</v>
+      </c>
+      <c r="F9" s="12">
         <v>48</v>
       </c>
-      <c r="G9" s="7">
-        <v>0</v>
-      </c>
-      <c r="H9" s="7">
-        <v>0</v>
-      </c>
-      <c r="I9" s="7">
-        <v>0</v>
-      </c>
-      <c r="J9" s="7">
+      <c r="G9" s="12">
+        <v>0</v>
+      </c>
+      <c r="H9" s="12">
+        <v>0</v>
+      </c>
+      <c r="I9" s="12">
+        <v>0</v>
+      </c>
+      <c r="J9" s="12">
         <v>18</v>
       </c>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7">
+      <c r="K9" s="12"/>
+      <c r="L9" s="12">
         <v>150</v>
       </c>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7">
-        <v>517</v>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12">
+        <f>IFERROR(C9+K9+(SUM(D9,F9,H9)*3)+(SUM(E9,G9,I9)*2)+(J9*4),"")</f>
+        <v>235</v>
       </c>
     </row>
     <row r="10" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="12">
         <v>2</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="12">
         <v>12</v>
       </c>
-      <c r="E10" s="7">
-        <v>0</v>
-      </c>
-      <c r="F10" s="7">
-        <v>0</v>
-      </c>
-      <c r="G10" s="7">
-        <v>0</v>
-      </c>
-      <c r="H10" s="7">
-        <v>0</v>
-      </c>
-      <c r="I10" s="7">
-        <v>0</v>
-      </c>
-      <c r="J10" s="7">
-        <v>0</v>
-      </c>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7">
-        <v>0</v>
-      </c>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7">
-        <v>46</v>
+      <c r="E10" s="12">
+        <v>0</v>
+      </c>
+      <c r="F10" s="12">
+        <v>0</v>
+      </c>
+      <c r="G10" s="12">
+        <v>0</v>
+      </c>
+      <c r="H10" s="12">
+        <v>0</v>
+      </c>
+      <c r="I10" s="12">
+        <v>0</v>
+      </c>
+      <c r="J10" s="12">
+        <v>0</v>
+      </c>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12">
+        <v>0</v>
+      </c>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12">
+        <f t="shared" ref="N10:N27" si="0">IFERROR(C10+K10+(SUM(D10,F10,H10)*3)+(SUM(E10,G10,I10)*2)+(J10*4),"")</f>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="7">
-        <v>0</v>
-      </c>
-      <c r="D11" s="7">
-        <v>0</v>
-      </c>
-      <c r="E11" s="7">
-        <v>0</v>
-      </c>
-      <c r="F11" s="7">
-        <v>0</v>
-      </c>
-      <c r="G11" s="7">
-        <v>0</v>
-      </c>
-      <c r="H11" s="7">
+      <c r="C11" s="12">
+        <v>0</v>
+      </c>
+      <c r="D11" s="12">
+        <v>0</v>
+      </c>
+      <c r="E11" s="12">
+        <v>0</v>
+      </c>
+      <c r="F11" s="12">
+        <v>0</v>
+      </c>
+      <c r="G11" s="12">
+        <v>0</v>
+      </c>
+      <c r="H11" s="12">
         <v>3</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="12">
         <v>3</v>
       </c>
-      <c r="J11" s="7">
-        <v>0</v>
-      </c>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7">
-        <v>0</v>
-      </c>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7">
+      <c r="J11" s="12">
+        <v>0</v>
+      </c>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12">
+        <v>0</v>
+      </c>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
     </row>
@@ -831,110 +838,113 @@
       <c r="B12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="7">
-        <v>0</v>
-      </c>
-      <c r="D12" s="7">
-        <v>0</v>
-      </c>
-      <c r="E12" s="7">
-        <v>0</v>
-      </c>
-      <c r="F12" s="7">
+      <c r="C12" s="12">
+        <v>0</v>
+      </c>
+      <c r="D12" s="12">
+        <v>0</v>
+      </c>
+      <c r="E12" s="12">
+        <v>0</v>
+      </c>
+      <c r="F12" s="12">
         <v>3</v>
       </c>
-      <c r="G12" s="7">
-        <v>0</v>
-      </c>
-      <c r="H12" s="7">
-        <v>0</v>
-      </c>
-      <c r="I12" s="7">
-        <v>0</v>
-      </c>
-      <c r="J12" s="7">
-        <v>0</v>
-      </c>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7">
+      <c r="G12" s="12">
+        <v>0</v>
+      </c>
+      <c r="H12" s="12">
+        <v>0</v>
+      </c>
+      <c r="I12" s="12">
+        <v>0</v>
+      </c>
+      <c r="J12" s="12">
+        <v>0</v>
+      </c>
+      <c r="K12" s="12"/>
+      <c r="L12" s="12">
         <v>5</v>
       </c>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7">
-        <v>14</v>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12">
+        <f t="shared" si="0"/>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="12">
         <v>1</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="12">
         <v>12</v>
       </c>
-      <c r="E13" s="7">
-        <v>0</v>
-      </c>
-      <c r="F13" s="7">
+      <c r="E13" s="12">
+        <v>0</v>
+      </c>
+      <c r="F13" s="12">
         <v>20</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="12">
         <v>40</v>
       </c>
-      <c r="H13" s="7">
-        <v>0</v>
-      </c>
-      <c r="I13" s="7">
-        <v>0</v>
-      </c>
-      <c r="J13" s="7">
-        <v>0</v>
-      </c>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7">
+      <c r="H13" s="12">
+        <v>0</v>
+      </c>
+      <c r="I13" s="12">
+        <v>0</v>
+      </c>
+      <c r="J13" s="12">
+        <v>0</v>
+      </c>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12">
         <v>50</v>
       </c>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7">
-        <v>407</v>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12">
+        <f t="shared" si="0"/>
+        <v>177</v>
       </c>
     </row>
     <row r="14" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="7">
-        <v>0</v>
-      </c>
-      <c r="D14" s="7">
-        <v>0</v>
-      </c>
-      <c r="E14" s="7">
-        <v>0</v>
-      </c>
-      <c r="F14" s="7">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7">
-        <v>0</v>
-      </c>
-      <c r="H14" s="7">
-        <v>0</v>
-      </c>
-      <c r="I14" s="7">
-        <v>0</v>
-      </c>
-      <c r="J14" s="7">
+      <c r="C14" s="12">
+        <v>0</v>
+      </c>
+      <c r="D14" s="12">
+        <v>0</v>
+      </c>
+      <c r="E14" s="12">
+        <v>0</v>
+      </c>
+      <c r="F14" s="12">
+        <v>0</v>
+      </c>
+      <c r="G14" s="12">
+        <v>0</v>
+      </c>
+      <c r="H14" s="12">
+        <v>0</v>
+      </c>
+      <c r="I14" s="12">
+        <v>0</v>
+      </c>
+      <c r="J14" s="12">
         <v>3</v>
       </c>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7">
-        <v>0</v>
-      </c>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7">
+      <c r="K14" s="12"/>
+      <c r="L14" s="12">
+        <v>0</v>
+      </c>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
     </row>
@@ -942,36 +952,37 @@
       <c r="B15" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="7">
-        <v>0</v>
-      </c>
-      <c r="D15" s="7">
-        <v>0</v>
-      </c>
-      <c r="E15" s="7">
-        <v>0</v>
-      </c>
-      <c r="F15" s="7">
+      <c r="C15" s="12">
+        <v>0</v>
+      </c>
+      <c r="D15" s="12">
+        <v>0</v>
+      </c>
+      <c r="E15" s="12">
+        <v>0</v>
+      </c>
+      <c r="F15" s="12">
         <v>4</v>
       </c>
-      <c r="G15" s="7">
-        <v>0</v>
-      </c>
-      <c r="H15" s="7">
+      <c r="G15" s="12">
+        <v>0</v>
+      </c>
+      <c r="H15" s="12">
         <v>3</v>
       </c>
-      <c r="I15" s="7">
-        <v>0</v>
-      </c>
-      <c r="J15" s="7">
-        <v>0</v>
-      </c>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7">
-        <v>0</v>
-      </c>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7">
+      <c r="I15" s="12">
+        <v>0</v>
+      </c>
+      <c r="J15" s="12">
+        <v>0</v>
+      </c>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12">
+        <v>0</v>
+      </c>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
     </row>
@@ -979,36 +990,37 @@
       <c r="B16" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="7">
-        <v>0</v>
-      </c>
-      <c r="D16" s="7">
-        <v>0</v>
-      </c>
-      <c r="E16" s="7">
-        <v>0</v>
-      </c>
-      <c r="F16" s="7">
+      <c r="C16" s="12">
+        <v>0</v>
+      </c>
+      <c r="D16" s="12">
+        <v>0</v>
+      </c>
+      <c r="E16" s="12">
+        <v>0</v>
+      </c>
+      <c r="F16" s="12">
         <v>3</v>
       </c>
-      <c r="G16" s="7">
-        <v>0</v>
-      </c>
-      <c r="H16" s="7">
-        <v>0</v>
-      </c>
-      <c r="I16" s="7">
-        <v>0</v>
-      </c>
-      <c r="J16" s="7">
-        <v>0</v>
-      </c>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7">
-        <v>0</v>
-      </c>
-      <c r="M16" s="7"/>
-      <c r="N16" s="7">
+      <c r="G16" s="12">
+        <v>0</v>
+      </c>
+      <c r="H16" s="12">
+        <v>0</v>
+      </c>
+      <c r="I16" s="12">
+        <v>0</v>
+      </c>
+      <c r="J16" s="12">
+        <v>0</v>
+      </c>
+      <c r="K16" s="12"/>
+      <c r="L16" s="12">
+        <v>0</v>
+      </c>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
@@ -1016,36 +1028,37 @@
       <c r="B17" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="7">
-        <v>0</v>
-      </c>
-      <c r="D17" s="7">
+      <c r="C17" s="12">
+        <v>0</v>
+      </c>
+      <c r="D17" s="12">
         <v>4</v>
       </c>
-      <c r="E17" s="7">
-        <v>0</v>
-      </c>
-      <c r="F17" s="7">
+      <c r="E17" s="12">
+        <v>0</v>
+      </c>
+      <c r="F17" s="12">
         <v>2</v>
       </c>
-      <c r="G17" s="7">
-        <v>0</v>
-      </c>
-      <c r="H17" s="7">
+      <c r="G17" s="12">
+        <v>0</v>
+      </c>
+      <c r="H17" s="12">
         <v>3</v>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="12">
         <v>3</v>
       </c>
-      <c r="J17" s="7">
-        <v>0</v>
-      </c>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7">
-        <v>0</v>
-      </c>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7">
+      <c r="J17" s="12">
+        <v>0</v>
+      </c>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12">
+        <v>0</v>
+      </c>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12">
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
     </row>
@@ -1053,352 +1066,365 @@
       <c r="B18" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="7">
-        <v>0</v>
-      </c>
-      <c r="D18" s="7">
+      <c r="C18" s="12">
+        <v>0</v>
+      </c>
+      <c r="D18" s="12">
         <v>6</v>
       </c>
-      <c r="E18" s="7">
-        <v>0</v>
-      </c>
-      <c r="F18" s="7">
+      <c r="E18" s="12">
+        <v>0</v>
+      </c>
+      <c r="F18" s="12">
         <v>4</v>
       </c>
-      <c r="G18" s="7">
-        <v>0</v>
-      </c>
-      <c r="H18" s="7">
-        <v>0</v>
-      </c>
-      <c r="I18" s="7">
-        <v>0</v>
-      </c>
-      <c r="J18" s="7">
-        <v>0</v>
-      </c>
-      <c r="K18" s="7"/>
-      <c r="L18" s="7">
+      <c r="G18" s="12">
+        <v>0</v>
+      </c>
+      <c r="H18" s="12">
+        <v>0</v>
+      </c>
+      <c r="I18" s="12">
+        <v>0</v>
+      </c>
+      <c r="J18" s="12">
+        <v>0</v>
+      </c>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12">
         <v>5</v>
       </c>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7">
-        <v>35</v>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12">
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="J19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="K19" s="7"/>
-      <c r="L19" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M19" s="7"/>
-      <c r="N19" s="7" t="s">
-        <v>16</v>
+      <c r="C19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v/>
       </c>
     </row>
     <row r="20" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="K20" s="7"/>
-      <c r="L20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M20" s="7"/>
-      <c r="N20" s="7" t="s">
-        <v>16</v>
+      <c r="C20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v/>
       </c>
     </row>
     <row r="21" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="J21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7" t="s">
-        <v>16</v>
+      <c r="C21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v/>
       </c>
     </row>
     <row r="22" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="J22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="K22" s="7"/>
-      <c r="L22" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M22" s="7"/>
-      <c r="N22" s="7" t="s">
-        <v>16</v>
+      <c r="C22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K22" s="12"/>
+      <c r="L22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v/>
       </c>
     </row>
     <row r="23" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="J23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7" t="s">
-        <v>16</v>
+      <c r="C23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v/>
       </c>
     </row>
     <row r="24" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="J24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7" t="s">
-        <v>16</v>
+      <c r="C24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K24" s="12"/>
+      <c r="L24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v/>
       </c>
     </row>
     <row r="25" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="J25" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M25" s="7"/>
-      <c r="N25" s="7" t="s">
-        <v>16</v>
+      <c r="C25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v/>
       </c>
     </row>
     <row r="26" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="J26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M26" s="7"/>
-      <c r="N26" s="7" t="s">
-        <v>16</v>
+      <c r="C26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K26" s="12"/>
+      <c r="L26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v/>
       </c>
     </row>
     <row r="27" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="7"/>
-      <c r="N27" s="7"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update staff summry template
</commit_message>
<xml_diff>
--- a/XcelUnify/Data/staff-summary.xlsx
+++ b/XcelUnify/Data/staff-summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_work\melb\2025\safe\Application\XcelUnify\XcelUnify\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1FE73A-E430-4252-800C-8C5883DA3CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF786A78-CC87-46DE-B2B9-2012E896AFC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{D83A47D0-BE84-4F4B-BC6D-31D7CF1B83A6}"/>
+    <workbookView xWindow="38790" yWindow="0" windowWidth="19200" windowHeight="15480" xr2:uid="{D83A47D0-BE84-4F4B-BC6D-31D7CF1B83A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="32">
   <si>
     <t>Name</t>
   </si>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t>SUBJECT10</t>
+  </si>
+  <si>
+    <t>&lt;&lt;update, please&gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -638,31 +641,31 @@
       <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="10">
-        <v>1</v>
+      <c r="C3" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="2:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="10">
-        <v>2</v>
+      <c r="C4" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="2:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="10">
-        <v>3</v>
+      <c r="C5" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>4</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="H5" s="8">
-        <v>100</v>
+      <c r="H5" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.25">
@@ -679,6 +682,9 @@
       <c r="K7" s="11"/>
       <c r="L7" s="3" t="s">
         <v>6</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="2:14" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>